<commit_message>
Fix EBITDA 2024 discrepancy and update benchmarking
</commit_message>
<xml_diff>
--- a/model/Dialog_Axiata_Financial_Model.xlsx
+++ b/model/Dialog_Axiata_Financial_Model.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dialog axiata financial Analyst\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dialog axiata financial Analyst\model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C613AC6-40F8-4848-A1D0-C1E896DA7EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AB21B41-30D5-4679-B960-223EB0EA766F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions" sheetId="1" r:id="rId1"/>
@@ -829,15 +829,33 @@
     <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="166" fontId="10" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -847,30 +865,30 @@
     <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -878,24 +896,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1175,42 +1175,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
     </row>
     <row r="3" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="53" t="s">
+      <c r="B3" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="53" t="s">
+      <c r="C3" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="53" t="s">
+      <c r="D3" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="53" t="s">
+      <c r="E3" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="53" t="s">
+      <c r="F3" s="45" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1223,14 +1223,14 @@
       <c r="F4" s="44"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="49" t="s">
+      <c r="A5" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="49"/>
-      <c r="C5" s="49"/>
-      <c r="D5" s="49"/>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
+      <c r="B5" s="46"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
@@ -1338,24 +1338,24 @@
       </c>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="50" t="s">
+      <c r="A11" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="50"/>
-      <c r="C11" s="50"/>
-      <c r="D11" s="50"/>
-      <c r="E11" s="50"/>
-      <c r="F11" s="50"/>
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="49" t="s">
+      <c r="A13" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="49"/>
-      <c r="C13" s="49"/>
-      <c r="D13" s="49"/>
-      <c r="E13" s="49"/>
-      <c r="F13" s="49"/>
+      <c r="B13" s="46"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="46"/>
+      <c r="E13" s="46"/>
+      <c r="F13" s="46"/>
     </row>
     <row r="14" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
@@ -1463,24 +1463,24 @@
       </c>
     </row>
     <row r="19" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="50" t="s">
+      <c r="A19" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="50"/>
-      <c r="C19" s="50"/>
-      <c r="D19" s="50"/>
-      <c r="E19" s="50"/>
-      <c r="F19" s="50"/>
+      <c r="B19" s="47"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="47"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="47"/>
     </row>
     <row r="21" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="49" t="s">
+      <c r="A21" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="49"/>
-      <c r="C21" s="49"/>
-      <c r="D21" s="49"/>
-      <c r="E21" s="49"/>
-      <c r="F21" s="49"/>
+      <c r="B21" s="46"/>
+      <c r="C21" s="46"/>
+      <c r="D21" s="46"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="46"/>
     </row>
     <row r="22" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
@@ -1531,10 +1531,10 @@
       <c r="A27" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="43">
+      <c r="B27" s="50">
         <v>6.5</v>
       </c>
-      <c r="C27" s="43"/>
+      <c r="C27" s="50"/>
     </row>
     <row r="29" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="44" t="s">
@@ -1547,47 +1547,63 @@
       <c r="F29" s="44"/>
     </row>
     <row r="30" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="45" t="s">
+      <c r="A30" s="51" t="s">
         <v>30</v>
       </c>
-      <c r="B30" s="45"/>
-      <c r="C30" s="45"/>
-      <c r="D30" s="45"/>
-      <c r="E30" s="45"/>
-      <c r="F30" s="45"/>
+      <c r="B30" s="51"/>
+      <c r="C30" s="51"/>
+      <c r="D30" s="51"/>
+      <c r="E30" s="51"/>
+      <c r="F30" s="51"/>
     </row>
     <row r="31" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="46" t="s">
+      <c r="A31" s="52" t="s">
         <v>31</v>
       </c>
-      <c r="B31" s="46"/>
-      <c r="C31" s="46"/>
-      <c r="D31" s="46"/>
-      <c r="E31" s="46"/>
-      <c r="F31" s="46"/>
+      <c r="B31" s="52"/>
+      <c r="C31" s="52"/>
+      <c r="D31" s="52"/>
+      <c r="E31" s="52"/>
+      <c r="F31" s="52"/>
     </row>
     <row r="32" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="53" t="s">
         <v>32</v>
       </c>
-      <c r="B32" s="47"/>
-      <c r="C32" s="47"/>
-      <c r="D32" s="47"/>
-      <c r="E32" s="47"/>
-      <c r="F32" s="47"/>
+      <c r="B32" s="53"/>
+      <c r="C32" s="53"/>
+      <c r="D32" s="53"/>
+      <c r="E32" s="53"/>
+      <c r="F32" s="53"/>
     </row>
     <row r="33" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="42" t="s">
+      <c r="A33" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="B33" s="42"/>
-      <c r="C33" s="42"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="42"/>
-      <c r="F33" s="42"/>
+      <c r="B33" s="49"/>
+      <c r="C33" s="49"/>
+      <c r="D33" s="49"/>
+      <c r="E33" s="49"/>
+      <c r="F33" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A21:F21"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:A4"/>
@@ -1596,22 +1612,6 @@
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="A33:F33"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A32:F32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1641,16 +1641,16 @@
       <c r="H1" s="54"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
     </row>
     <row r="3" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9"/>
@@ -2036,15 +2036,15 @@
       <c r="G1" s="54"/>
     </row>
     <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="43" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
     </row>
     <row r="3" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -2070,15 +2070,15 @@
       </c>
     </row>
     <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="46" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="49"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
     </row>
     <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
@@ -2173,15 +2173,15 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="49" t="s">
+      <c r="A9" s="46" t="s">
         <v>64</v>
       </c>
-      <c r="B9" s="49"/>
-      <c r="C9" s="49"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="49"/>
+      <c r="B9" s="46"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
     </row>
     <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -2293,15 +2293,15 @@
       </c>
     </row>
     <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="49" t="s">
+      <c r="A15" s="46" t="s">
         <v>72</v>
       </c>
-      <c r="B15" s="49"/>
-      <c r="C15" s="49"/>
-      <c r="D15" s="49"/>
-      <c r="E15" s="49"/>
-      <c r="F15" s="49"/>
-      <c r="G15" s="49"/>
+      <c r="B15" s="46"/>
+      <c r="C15" s="46"/>
+      <c r="D15" s="46"/>
+      <c r="E15" s="46"/>
+      <c r="F15" s="46"/>
+      <c r="G15" s="46"/>
     </row>
     <row r="16" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
@@ -2425,30 +2425,30 @@
       <c r="I1" s="54"/>
     </row>
     <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="43" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52"/>
-      <c r="I2" s="52"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
     </row>
     <row r="4" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="46" t="s">
         <v>80</v>
       </c>
-      <c r="B4" s="49"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
-      <c r="H4" s="49"/>
-      <c r="I4" s="49"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="46"/>
+      <c r="I4" s="46"/>
     </row>
     <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="28" t="s">
@@ -2550,21 +2550,21 @@
     </row>
     <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="33"/>
-      <c r="B13" s="62" t="s">
+      <c r="B13" s="56" t="s">
         <v>90</v>
       </c>
-      <c r="C13" s="62"/>
-      <c r="D13" s="62"/>
-      <c r="E13" s="63" t="s">
+      <c r="C13" s="56"/>
+      <c r="D13" s="56"/>
+      <c r="E13" s="57" t="s">
         <v>91</v>
       </c>
-      <c r="F13" s="63"/>
-      <c r="G13" s="63"/>
-      <c r="H13" s="64" t="s">
+      <c r="F13" s="57"/>
+      <c r="G13" s="57"/>
+      <c r="H13" s="58" t="s">
         <v>92</v>
       </c>
-      <c r="I13" s="64"/>
-      <c r="J13" s="64"/>
+      <c r="I13" s="58"/>
+      <c r="J13" s="58"/>
     </row>
     <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="33"/>
@@ -2737,37 +2737,37 @@
       </c>
     </row>
     <row r="21" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="49" t="s">
+      <c r="A21" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="B21" s="49"/>
-      <c r="C21" s="49"/>
-      <c r="D21" s="49"/>
-      <c r="E21" s="49"/>
-      <c r="F21" s="49"/>
-      <c r="G21" s="49"/>
-      <c r="H21" s="49"/>
-      <c r="I21" s="49"/>
+      <c r="B21" s="46"/>
+      <c r="C21" s="46"/>
+      <c r="D21" s="46"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="46"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="46"/>
+      <c r="I21" s="46"/>
     </row>
     <row r="22" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B22" s="61">
+      <c r="B22" s="59">
         <v>155112</v>
       </c>
-      <c r="C22" s="61"/>
-      <c r="D22" s="61"/>
-      <c r="E22" s="61">
+      <c r="C22" s="59"/>
+      <c r="D22" s="59"/>
+      <c r="E22" s="59">
         <v>97938</v>
       </c>
-      <c r="F22" s="61"/>
-      <c r="G22" s="61"/>
-      <c r="H22" s="61">
+      <c r="F22" s="59"/>
+      <c r="G22" s="59"/>
+      <c r="H22" s="59">
         <v>49895</v>
       </c>
-      <c r="I22" s="61"/>
-      <c r="J22" s="61"/>
+      <c r="I22" s="59"/>
+      <c r="J22" s="59"/>
     </row>
     <row r="23" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
@@ -2793,21 +2793,21 @@
       <c r="A24" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="B24" s="59">
+      <c r="B24" s="61">
         <v>692834</v>
       </c>
-      <c r="C24" s="59"/>
-      <c r="D24" s="59"/>
-      <c r="E24" s="59">
+      <c r="C24" s="61"/>
+      <c r="D24" s="61"/>
+      <c r="E24" s="61">
         <v>294144</v>
       </c>
-      <c r="F24" s="59"/>
-      <c r="G24" s="59"/>
-      <c r="H24" s="59">
+      <c r="F24" s="61"/>
+      <c r="G24" s="61"/>
+      <c r="H24" s="61">
         <v>116967</v>
       </c>
-      <c r="I24" s="59"/>
-      <c r="J24" s="59"/>
+      <c r="I24" s="61"/>
+      <c r="J24" s="61"/>
     </row>
     <row r="25" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
@@ -2833,63 +2833,70 @@
       <c r="A26" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="B26" s="57">
+      <c r="B26" s="63">
         <v>618926</v>
       </c>
-      <c r="C26" s="57"/>
-      <c r="D26" s="57"/>
-      <c r="E26" s="57">
+      <c r="C26" s="63"/>
+      <c r="D26" s="63"/>
+      <c r="E26" s="63">
         <v>220236</v>
       </c>
-      <c r="F26" s="57"/>
-      <c r="G26" s="57"/>
-      <c r="H26" s="57">
+      <c r="F26" s="63"/>
+      <c r="G26" s="63"/>
+      <c r="H26" s="63">
         <v>43059</v>
       </c>
-      <c r="I26" s="57"/>
-      <c r="J26" s="57"/>
+      <c r="I26" s="63"/>
+      <c r="J26" s="63"/>
     </row>
     <row r="27" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="B27" s="58">
+      <c r="B27" s="64">
         <v>75.48</v>
       </c>
-      <c r="C27" s="58"/>
-      <c r="D27" s="58"/>
-      <c r="E27" s="58">
+      <c r="C27" s="64"/>
+      <c r="D27" s="64"/>
+      <c r="E27" s="64">
         <v>26.86</v>
       </c>
-      <c r="F27" s="58"/>
-      <c r="G27" s="58"/>
-      <c r="H27" s="58">
+      <c r="F27" s="64"/>
+      <c r="G27" s="64"/>
+      <c r="H27" s="64">
         <v>5.25</v>
       </c>
-      <c r="I27" s="58"/>
-      <c r="J27" s="58"/>
+      <c r="I27" s="64"/>
+      <c r="J27" s="64"/>
     </row>
     <row r="29" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="56" t="s">
+      <c r="A29" s="62" t="s">
         <v>109</v>
       </c>
-      <c r="B29" s="56"/>
-      <c r="C29" s="56"/>
-      <c r="D29" s="56"/>
-      <c r="E29" s="56"/>
-      <c r="F29" s="56"/>
-      <c r="G29" s="56"/>
-      <c r="H29" s="56"/>
-      <c r="I29" s="56"/>
+      <c r="B29" s="62"/>
+      <c r="C29" s="62"/>
+      <c r="D29" s="62"/>
+      <c r="E29" s="62"/>
+      <c r="F29" s="62"/>
+      <c r="G29" s="62"/>
+      <c r="H29" s="62"/>
+      <c r="I29" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="H26:J26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="H24:J24"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="H25:J25"/>
     <mergeCell ref="A21:I21"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="E22:G22"/>
@@ -2897,19 +2904,12 @@
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="E23:G23"/>
     <mergeCell ref="H23:J23"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="H24:J24"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="H25:J25"/>
-    <mergeCell ref="A29:I29"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="H26:J26"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="H13:J13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2937,15 +2937,15 @@
       <c r="G1" s="54"/>
     </row>
     <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="43" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
     </row>
     <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9"/>
@@ -3054,7 +3054,7 @@
         <v>61918</v>
       </c>
       <c r="F7" s="41">
-        <v>66275</v>
+        <v>66276</v>
       </c>
       <c r="G7" s="36">
         <v>282299</v>

</xml_diff>